<commit_message>
vault backup: 2026-06-28 23:00:16
Affected files:
_inbox/从会员运营到toc全面数字化：2023中国零售业会员运营报告-中国百货商业协会.pdf
demo/五技能演示/01-求职分析笔记.md
wiki/career/求职/岗位汇总_2026-06-28_综合排序_v7.xlsx
wiki/career/求职/岗位汇总_v7_总表.md
wiki/career/调研/7家投递优先级+行动清单.md
</commit_message>
<xml_diff>
--- a/wiki/career/求职/岗位汇总_2026-06-28_综合排序_v7.xlsx
+++ b/wiki/career/求职/岗位汇总_2026-06-28_综合排序_v7.xlsx
@@ -3847,8 +3847,6 @@
           <t>✅高匹配</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>广州·天河·珠江新城</t>
@@ -3856,13 +3854,17 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>✅双休</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
+          <t>✅双休 09:00-18:15</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>✅六险一金+包早晚餐下午茶+每年2次加薪+14薪+加班补贴</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>国货TOP·六险一金·包三餐·每年2次加薪·A轮高新</t>
+          <t>✅低风险 — 私企(A轮·100-499人·高新企业)·非上市·非外企，不会深度背调</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -3915,8 +3917,6 @@
           <t>✅高匹配</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>广州·天河·林和</t>
@@ -3924,13 +3924,17 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>✅双休</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
+          <t>✅双休（行业推测，未明确标注）</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>❓未明确</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>服装CRM·会员体系搭建+服饰零售3年双重覆盖</t>
+          <t>✅低风险 — 私企·非上市·服装行业正规企业，不会深度背调</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -4010,7 +4014,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>中等-中大型培训机构(1000-9999人),管理岗可能做正规背调</t>
+          <t>🟡中等风险 — 中大型培训机构(1000-9999人)，管理岗可能做正规背调 ⚡可能第三方</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -4063,8 +4067,6 @@
           <t>✅高匹配</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>广州·天河·天平架</t>
@@ -4072,13 +4074,17 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>✅双休</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
+          <t>✅双休（办公室岗7小时）</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>✅五险一金+年终奖金+绩效奖金+技能培训+岗位晋升</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>养老龙头2000+人·JD最全面·办公室岗7小时双休</t>
+          <t>✅低风险 — 私企(2000-5000人)·省级养老龙头·非上市/外企</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -4148,17 +4154,17 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>❓待确认</t>
+          <t>⚠️大小周（服装行业常见）</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>✅五险一金</t>
+          <t>✅五险一金+补充医疗+年终奖+定期体检</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>轻时尚男装200+店⚠️大小周(确认)</t>
+          <t>✅低风险 — 私企(500-999人)·不需要融资，不会深度背调</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -4211,8 +4217,6 @@
           <t>✅高匹配</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>广州·琶洲·欢聚大厦</t>
@@ -4220,13 +4224,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>✅双休</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr"/>
+          <t>✅弹性工作</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>✅五险一金+绩效奖金+扁平管理+弹性工作+内购福利</t>
+        </is>
+      </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>集团A轮+中科院合作·1-49人极低背调风险·扁平管理</t>
+          <t>✅极低风险 — 1-49人极小私企，几乎不做背调</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -4279,8 +4287,6 @@
           <t>✅高匹配</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>天河·广州银行大厦</t>
@@ -4291,10 +4297,14 @@
           <t>✅双休</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>🟡绩效奖金（其他未明确）</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>高端服装·8.1分好评(74%好评)·在招110岗业务扩张</t>
+          <t>✅低风险 — 私企未上市(500-1000人)，不会深度背调</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -4369,12 +4379,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>🟡仅五险</t>
+          <t>🟡仅五险+包食宿</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>民企餐饮连锁·低背调风险·包食宿</t>
+          <t>✅低风险 — 民企餐饮连锁(1000-9999人)·未融资 ✓经核实</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -4427,8 +4437,6 @@
           <t>✅高匹配</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>广州·海珠·新港</t>
@@ -4436,13 +4444,17 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>✅双休</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr"/>
+          <t>✅双休（大促加班）</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>✅五险一金+带薪年假+岗位晋升+节日礼物</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>新式滋补花胶TOP·月GMV 300-500万+·低背调·确认职级</t>
+          <t>✅低风险 — 私企(500-999人)·新式滋补TOP·非上市</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -4522,7 +4534,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>低(100-499人文化电商)</t>
+          <t>✅低风险 — 100-499人文化电商·未融资 ✓经核实</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4575,8 +4587,6 @@
           <t>🟡中匹配</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>广州·天河·珠江新城</t>
@@ -4587,10 +4597,14 @@
           <t>❓待确认</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>❓未明确</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>天使轮100-499人·偏社群裂变方向</t>
+          <t>✅低风险 — 天使轮100-499人·金融科技·非上市</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -4693,7 +4707,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>⚠️医美行业需补课·员工评分4.4但合规风险(高潮针被央视曝光)</t>
+          <t>🟡中等风险 — 正规企业注册资本3.6亿·2008年成立 ⚡可能第三方背调</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -4853,7 +4867,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>低(100-499人电商)</t>
+          <t>待确认</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -4933,7 +4947,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>低(100-499人日化)·薪资最高档·白云略远</t>
+          <t>✅低风险 — 私企(100-499人日化)·不需要融资 ✓经核实</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -5146,8 +5160,6 @@
           <t>🟡中匹配</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>广州·越秀·建设路</t>
@@ -5155,13 +5167,17 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>❓待确认</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr"/>
+          <t>✅双休 09:00-18:30</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>✅五险一金+补充医疗+绩效奖金+晋升机制</t>
+        </is>
+      </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>C轮·双休·需确认汽配经验要求·加班偏多</t>
+          <t>✅低风险 — C轮私企(100-499人)，不会做第三方深度背调</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -5214,8 +5230,6 @@
           <t>🟡中匹配</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>广州·天河·冼村</t>
@@ -5223,13 +5237,17 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>❓待确认</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr"/>
+          <t>✅双休 09:30-18:30</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>✅五险一金+餐补+交通补助+通讯补贴+下午茶+员工旅游</t>
+        </is>
+      </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>纳税A级+高新·20-99人极低背调·需补汽车营销知识</t>
+          <t>✅极低风险 — 小型私企(20-99人·参保29人)，几乎不做背调</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -7002,8 +7020,6 @@
           <t>✅高匹配</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
           <t>广州·海珠·新港</t>
@@ -7011,13 +7027,17 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>❓待确认</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr"/>
+          <t>❓待确认（大型集团通常双休）</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>✅五险一金+年终奖金+绩效奖金+补充医疗+定期体检</t>
+        </is>
+      </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>⚠️中外合营大型集团(2000-5000人)·背调待确认·8.3分好评</t>
+          <t>⚠️待确认 — 中外合营大型集团(2000-5000人)，面试时务必问清背调范围</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -7070,8 +7090,6 @@
           <t>✅高匹配</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>广州·越秀·时代地产中心</t>
@@ -7079,13 +7097,17 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>❓待确认</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr"/>
+          <t>✅双休 朝九晚六</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>✅五险一金</t>
+        </is>
+      </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>⚠️易展翅母公司·自营「展翅背调」品牌·背调待确认</t>
+          <t>⚠️高风险 — 集团旗下有自营「展翅背调」品牌，大概率会背调，面试确认范围</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -7165,7 +7187,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>低(100-499人电商)⚠️大小周</t>
+          <t>✅低风险 — 100-499人电商 ✓经核实</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -7218,8 +7240,6 @@
           <t>🟡中匹配</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>广州·黄埔·东圃</t>
@@ -7230,10 +7250,14 @@
           <t>❓待确认</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>🟡包餐（其他未明确）</t>
+        </is>
+      </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>1000-9999人·包餐·偏电商方向·大小周待确认</t>
+          <t>🟡待确认 — 千人规模(1000-9999人)，可能做正规背调</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -7286,8 +7310,6 @@
           <t>🟡中匹配</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>广州·海珠·赤岗</t>
@@ -7298,10 +7320,14 @@
           <t>❓待确认</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>❓未明确</t>
+        </is>
+      </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>⚠️90天前更新·网上零信息·待确认</t>
+          <t>⚠️待确认 — 网上零评价信息·90天前更新，需进一步了解</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -7381,7 +7407,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>千人规模可能背调·下降级</t>
+          <t>待确认</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -7434,8 +7460,6 @@
           <t>🟡中匹配</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>广州·海珠·乐天智谷</t>
@@ -7446,10 +7470,14 @@
           <t>❓待确认</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>❓未明确</t>
+        </is>
+      </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>无口碑数据·总监title可能inflation</t>
+          <t>⚠️待确认 — 网上零口碑数据，需先了解产品和公司实际规模</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -7502,8 +7530,6 @@
           <t>🟡中匹配</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>广州·越秀·华乐</t>
@@ -7511,13 +7537,17 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>❓待确认</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr"/>
+          <t>✅双休 09:00-18:30</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>✅入职即买社保+试用期全额</t>
+        </is>
+      </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>⚠️招聘缩85%+JD与主业不符(写车辆全生命周期)</t>
+          <t>⚠️存疑 — 2025招聘需求较2024降85%，JD与主营不符(车辆生命周期)，需防岗位包装</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">

</xml_diff>